<commit_message>
inventory auto update test
</commit_message>
<xml_diff>
--- a/Blackwood_CFS_Master_Inventory.xlsx
+++ b/Blackwood_CFS_Master_Inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\OneDrive\HOME\Documents\GitHub\Blackwood-CFS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA10522D-1361-467B-8005-0D6907310CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE1E814-09F6-45FC-B481-3E6AAE67E1F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2619" uniqueCount="927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2620" uniqueCount="928">
   <si>
     <t>Item_ID</t>
   </si>
@@ -2981,6 +2981,9 @@
 Clock
 Entry Control sheets
 (Keyword: Breathing Apparatus)</t>
+  </si>
+  <si>
+    <t>Test Edit.</t>
   </si>
 </sst>
 </file>
@@ -3387,7 +3390,9 @@
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="I2" s="5" t="s">
+        <v>927</v>
+      </c>
       <c r="J2" s="5" t="s">
         <v>14</v>
       </c>

</xml_diff>